<commit_message>
feat(kmp): add :shared module + iOS scaffold; remove voice commands
- ORDER-P0-001: :shared KMP module (AGP 9 KMP library plugin), XcodeGen iOS shell,
  Gradle memory fix (daemon strategy, 4g/3g on a 16 GB box), ASCII rootProject.name
- ORDER-P0-006: voice-command feature removed per client cancellation
  (4 files deleted, 7 edited, RECORD_AUDIO and RecognitionService queries dropped)
- SpeechManager retained: it is TalkBack detection, not voice input

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H9h8cPrJnYtU5ZsmseaUnp
</commit_message>
<xml_diff>
--- a/.agents/HOOKS_GUIDE.xlsx
+++ b/.agents/HOOKS_GUIDE.xlsx
@@ -10,24 +10,28 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الملخص العام" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. خطاف البدء والافتتاح" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. خطاف هندسة السياق" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. خطاف الإشراف العام وتصحيح" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. خطاف خط الإنتاج البرمجي" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. خطاف التكامل الفني" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. خطاف تدقيق الصيانة" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. خطاف الفحص الأمني" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. خطاف مراجعة وتحديث المكتب" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. خطاف الفحص والاختبار التل" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. خطاف معالجة الأخطاء والأع" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. خطاف إدارة النسخ والمستود" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. خطاف تحديث الإنجازات" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. خطاف الذاكرة المستدامة" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14. خطاف النجاح والتحليل البع" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15. خطاف تنظيم وترتيب الأجهزة" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16. خطاف ترتيب الملفات لمسار " sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17. خطاف إدارة تليجرام" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18. خطاف التدقيق البرمجي الشا" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19. خطاف استكشاف وتكامل الموا" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20. خطاف المزامنة السحابية ال" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. خطاف التخصيص والتصدير الذ" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. خطاف الإشراف العام وتصحيح" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. خطاف خط الإنتاج البرمجي" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. خطاف التكامل الفني" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. خطاف تدقيق الصيانة" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. خطاف الفحص الأمني" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. خطاف مراجعة وتحديث المكتب" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. خطاف الفحص والاختبار التل" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. خطاف معالجة الأخطاء والأع" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. خطاف إدارة النسخ والمستود" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. خطاف تحديث الإنجازات" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14. خطاف الذاكرة المستدامة" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15. خطاف النجاح والتحليل البع" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16. خطاف تنظيم وترتيب الأجهزة" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17. خطاف ترتيب الملفات لمسار " sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18. خطاف إدارة تليجرام" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19. خطاف التدقيق البرمجي الشا" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20. خطاف استكشاف وتكامل الموا" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21. خطاف المزامنة السحابية وا" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22. خطاف قيادة وإدارة الأسطول" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23. خطاف تحويل وأتمتة سكربتات" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24. خطاف أتمتة مسارات العمل و" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -603,12 +607,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>3. خطاف الإشراف العام وتصحيح المسار</t>
+          <t>3. خطاف التخصيص والتصدير الذكي لطاقم المشروع</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
+          <t>اعتمد سياق المشروع, تخصيص وكلاء المشروع, تصدير بيئة المشروع, تخصيص الوكلاء</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -619,15 +623,55 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>[code-architect], [agent-optimizer], [prompt-engineer]</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>تحليل سياق المشروع وتصدير حزم الوكلاء محلياً مع التنظيف التلقائي (Pruning) وتوليد سكربت المزامنة.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **تحليل سياق المشروع المعتمد (`project_agent_tailor.py`):** فحص ملف `PROJECT_CONTEXT.md` واكتشاف حزم التقنيات المستخدمة (مثل: `android_compose`, `web`, `python_ai`, `construction_survey`).
+  2. **تصدير حزم الوكلاء والمهارات المطلوبة:** نسخ مهارات وبطاقات الوكلاء المتخصصين وحزمة النواة حصرياً إلى مجلد المشروع المحلي `.agents/`.
+  3. **التنظيف التلقائي الصارم للمهارات الفائضة (Pruning Engine):** مسح وحذف أي مهارات أو بطاقات وكلاء غير مستخدمة في المشروع المستهدف، لحماية نافذة السياق (Context Budget) من الهدر بنسبة 100%.
+  4. **توليد قالب المزامنة المحلي (`sync_local_agents.py`):** إنشاء سكربت خفيف داخل المشروع لتمكين المطور من تحديث طاقم المشروع بنقرة زر واحدة مستقبلاً دون المساس بخصوصية المشروع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>4. خطاف الإشراف العام وتصحيح المسار</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>[prompt-engineer], [agent-optimizer]</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>تصحيح الخطافات الخاطئة والبرومبتات غير الاحترافية وتوجيهها للمسار الصحيح تلقائياً.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
   1. **الرصد التلقائي والإيقاف:** يقوم الوكيل الرئيسي بمراقبة المحادثة. عند استخدام المستخدم لمحفز "تصحيح مسار"، أو عند رصد دخول وكيل في دائرة مفرغة، يتم اعتراض العمل وإيقافه فوراً.
@@ -637,85 +681,43 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>4. خطاف خط الإنتاج البرمجي</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [clean-code-guard], [android-testing], [test-guard]</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، حراسة الكود النظيف، والفحص والاختبار).</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>* **طريقة العمل والإجراءات:**
-  0. **حقن السياق الإجباري (Mandatory Context Injection):** يُلزم الوكيل الرئيسي بتشغيل أداة حقن السياق (`python .agents/inject_context.py`) وتمرير مخرجاتها كـ `System Alert` أو `&gt; [!WARNING] Mandatory Constraints` في المحادثة قبل بدء أي عمل.
-  1. **التصميم المعماري الهيكلي (`code-architect`):** يبدأ برسم معمارية الميزة وتحديد مواقع وتسمية الملفات الجديدة/المعدلة في الهيكل المناسب (Data/Domain/UI).
-  2. **التدقيق المعماري الصارم وحلقة الـ 7 مرات (7-Iterations Devil's Advocate Loop):** يُمنع منعاً باتاً البدء بكتابة الكود. يجب إدخال خطة التنفيذ (`implementation_plan.md`) في حلقة مراجعة وتدقيق مع "محامي الشيطان" **لـ 7 مرات متتالية** حتى يتم سد كل الثغرات والوصول لنسبة نجاح 99.99% وتأمين قسم `[UNINTENDED SIDE-EFFECTS &amp; LIFECYCLE HAZARDS]` بالكامل قبل السماح بالكتابة.
-  3. **الكتابة البرمجية (Surgical Precision Execution):** يستلم الوكيل `[android-kotlin-pro]` أو `[jetpack-compose-ui]` الخطة المعتمدة ويبدأ بالتنفيذ. **يُحقن الوكيل بالبرومبت الإجباري التالي:** *(يُمنع منعاً باتاً المساس، أو تعديل، أو حذف أي كود حالي في المشروع لا ينص عليه صراحة في خطة التنفيذ. تصرف كجراح دقيق: أضف ميزتك فقط دون إحداث أي تغييرات جانبية في الملفات المفتوحة).*
-  4. **المراجعة وحراسة الكود النظيف (`code-reviewer-quality` + `clean-code-guard`):** يفحص الكود بعد كتابته للتحقق من الاتساق، وخلوه من أخطاء الـ AI الـ 14 الشائعة (ابتلاع الأخطاء، تضخم الدوال، الأكواد المكررة).
-  5. **الأتمتة والاختبار النظيف (`android-testing` + `test-guard`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) وفق معايير `test-guard` للتحقق من سلوك النظام الفعلي وليس فقط الـ Happy Path، وتجنب الـ Mocks المفرطة.</t>
-        </is>
-      </c>
-    </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>5. خطاف التكامل الفني</t>
+          <t>5. خطاف خط الإنتاج البرمجي</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ربط API, تكامل خارجي</t>
+          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>[devops-deployer], [backend-architect]</t>
+          <t>[code-architect], [ui-ux-pro-max], [clean-code-guard], [test-guard]</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
+          <t>تنفيذ دورة التطوير الكاملة (المعمارية، الذكاء التصميمي، البرمجة، حراسة الكود النظيف، والفحص والاختبار).</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
-  2. **تحصين الانقطاع (API FAULT TOLERANCE CHECK):** يُمنع الدمج دون بناء `Interceptor` لمعالجة انقطاع الشبكة وإعادة المحاولة (Retry Mechanism)، وتغليف الردود بـ `Result&lt;T&gt;` أو `ErrorMapper` لمعالجة أخطاء HTTP (401, 404, 500).
-  3. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع وضمان التخزين المؤقت (Offline-First).
-  4. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
+  1. **التصميم الهيكلي والذكاء التصميمي (`code-architect` + `ui-ux-pro-max`):** تحديد المعمارية المناسبة، واستدعاء محرك الاستدلال التصميمي لتحديد نمط الواجهات (Style)، باليت الألوان الدلالية، والخطوط وقواعد سهولة الوصول بدقة قبل كتابة أي واجهة.
+  2. **التدقيق المعماري الصارم (Devil's Advocate Audit):** مراجعة الخطة وكشف الثغرات وحالات الحافة لمنع الآثار الجانبية.
+  3. **الكتابة البرمجية والتنفيذ:** كتابة الكود وبناء الواجهات وقواعد البيانات محلياً.
+  4. **المراجعة وضمان الجودة (`clean-code-guard` + `test-guard`):** فحص الكود للأمان، الأداء، والتوافق مع المعايير.</t>
         </is>
       </c>
     </row>
@@ -725,36 +727,36 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>6. خطاف تدقيق الصيانة</t>
+          <t>6. خطاف التكامل الفني</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>تدقيق صيانة, مراجعة DRY, كود نظيف</t>
+          <t>ربط API, تكامل خارجي</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [clean-code-guard], [performance-optimizer]</t>
+          <t>[devops-deployer], [backend-architect]</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية وتطبيق معايير الكود النظيف.</t>
+          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود النظيف والمكرر:** استدعاء الوكيل `[code-reviewer-quality]` و `[clean-code-guard]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY/KISS/YAGNI) والحد من التعقيد الحسابي.
-  2. **فحص Recomposition والأداء:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
-  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود وحذف الأكواد الميتة (Dead Code).</t>
+  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
+  2. **تحصين الانقطاع (API FAULT TOLERANCE CHECK):** بناء Interceptor لمعالجة انقطاع الشبكة وإعادة المحاولة وتأمين المفاتيح في متغيرات البيئة.
+  3. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.</t>
         </is>
       </c>
     </row>
@@ -764,36 +766,35 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7. خطاف الفحص الأمني</t>
+          <t>7. خطاف تدقيق الصيانة</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>فحص أمني, مراجعة أمان</t>
+          <t>تدقيق صيانة, مراجعة DRY, كود نظيف</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+ البديل: `Gemini 3.7 Flash (High)`</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>[security-auditor], [code-reviewer-quality]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [performance-optimizer]</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
+          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية وتطبيق معايير الكود النظيف.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest للبحث عن المكونات المكشوفة (`Exported=true`)، وتسريب البيانات عبر `Intents` (Intent Hijacking)، وقواعد `ProGuard`.
-  2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
-  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة و `SharedPreferences` والجلسات وحمايتها محلياً وسحابياً (إلزام إخراج تقرير يؤكد الفحص).</t>
+  1. **فحص الكود النظيف والمكرر:** استدعاء الوكيل `[code-reviewer-quality]` و `[clean-code-guard]` لمسح الملفات والتحقق من عدم وجود دوال مكررة (تطبيق DRY/KISS/YAGNI).
+  2. **فحص Recomposition والأداء:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.</t>
         </is>
       </c>
     </row>
@@ -803,44 +804,35 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>8. خطاف مراجعة وتحديث المكتبات والنماذج</t>
+          <t>8. خطاف الفحص الأمني</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>تحديث الاعتماديات, تحديث المكتبات, تحديث النماذج, معايرة النماذج, update models</t>
+          <t>فحص أمني, مراجعة أمان</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Gemini 3.6 Flash (Medium)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>[github-talent-scout], [code-architect], [agent-optimizer]</t>
+          <t>[security-auditor], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>فحص ملفات Gradle وتحديث المكتبات، والتحقق التلقائي عبر الإنترنت (antigravity.google) لتحديث مصفوفة النماذج ودليل hooks_user_guide.md دون لقطات شاشة.</t>
+          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص إصدارات المكتبات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
-  2. **الاستكشاف والمعايرة التلقائية للنماذج عبر الإنترنت (Online Model Discovery):**
-     - عند كتابة محفز `"تحديث النماذج"` أو `"معايرة النماذج"`، يقوم الوكيل `[agent-optimizer]` بالاستعلام الفوري عبر الإنترنت من المصادر الرسمية:
-       - 🌐 بوابة Google Antigravity الرسمية: `https://antigravity.google`
-       - 🌐 مدونة مطوري جوجل: `https://google.dev` و `https://blog.google`
-       - 🌐 دليل وثائق Anthropic: `https://docs.anthropic.com`
-     - يتم استخراج قائمة النماذج الفعالة في المحرر (مثل `Gemini 3.7 Flash`, `Claude Sonnet 4.6 (Thinking)`).
-  3. **التحديث والمزامنة الشاملة:**
-     - تحديث مصفوفة النماذج في `HOOKS_GUIDE.md` ودليل مسار العمل `hooks_user_guide.md`.
-     - تشغيل السكربتات لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx` وتطبيق مكتبة الأوامر HTML.
-     - تشغيل `sync_global_ecosystem.py` ورفع التحديثات لـ GitHub تلقائياً.</t>
+  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest والمكونات المكشوفة وتسريب البيانات.
+  2. **التحقق من صحة المدخلات وتشفير البيانات:** فحص تشفير البيانات الحساسة والجلسات وتأمين الوصول محلياً وسحابياً.</t>
         </is>
       </c>
     </row>
@@ -850,37 +842,35 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>9. خطاف الفحص والاختبار التلقائي</t>
+          <t>9. خطاف مراجعة وتحديث المكتبات والنماذج</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>قم بالاختبار, جاهز للتجربة</t>
+          <t>تحديث الاعتماديات, تحديث المكتبات, تحديث النماذج, معايرة النماذج, update models</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Gemini 3.6 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>[android-testing], [test-guard], [code-reviewer-quality]</t>
+          <t>[github-talent-scout], [code-architect], [agent-optimizer]</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>تشغيل اختبارات الوحدة وفحص جودة الكود واختبار السلوك الفعلي بدون Mock مفرط.</t>
+          <t>فحص ملفات Gradle وتحديث المكتبات، والتحقق التلقائي عبر الإنترنت (antigravity.google) لتحديث مصفوفة النماذج ودليل hooks_user_guide.md دون لقطات شاشة.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التقمص (Persona):** يتصرف الوكيل كمدير فحص جودة صارم (Pre-Flight Inspector &amp; Senior DevOps QA). بصرامة تامة وبدون أي مجاملات.
-  2. **حراسة الاختبارات (`test-guard`):** التحقق من أن الاختبارات تفحص سلوك النظام الفعلي ومخرجاته القابلة للملاحظة، ومنع الاختبارات الوهمية (Tautological Tests) والـ Mocks الزائدة.
-  3. **قاعدة التغطية الإجبارية (TEST COVERAGE MANDATE):** يُرفض أي اختبار يغطي مسار النجاح فقط (Happy Path). يجب كتابة اختبار للنجاح، الفشل، والحالات الطرفية (مثل: Network Off، Configuration Change).
-  4. **تقرير الفحص الصارم:** تزويد المطور بتقرير يحاكي المطالبة القياسية: `[BLOCKERS]`, `[WARNINGS]`, `[PRE-FLIGHT FIXES]`, `[GO / NO-GO]`.</t>
+  1. **فحص إصدارات المكتبات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
+  2. **الاستكشاف والمعايرة التلقائية للنماذج عبر الإنترنت (Online Model Discovery):** الاستعلام الفوري عبر المصادر الرسمية (antigravity.google, docs.anthropic.com) ومعايرة مصفوفة النماذج.</t>
         </is>
       </c>
     </row>
@@ -890,12 +880,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>10. خطاف معالجة الأخطاء والأعطال</t>
+          <t>10. خطاف الفحص والاختبار التلقائي</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>حدث خطأ, التطبيق توقف, Crash</t>
+          <t>قم بالاختبار, جاهز للتجربة</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -906,20 +896,19 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>[debugger]</t>
+          <t>[android-testing], [test-guard], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
+          <t>تشغيل اختبارات الوحدة وفحص جودة الكود واختبار السلوك الفعلي بدون Mock مفرط.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل.
-  2. **عزل المشكلة:** حصر الكود المسبب للأخطاء لمعرفة إن كان يتعلق بالشبكة، قاعدة البيانات، أو دورة حياة المكونات.
-  3. **اقتراح وتثبيت الحل:** تطبيق التعديل الأدنى الكافي لحل المشكلة مع حماية الأجزاء الأخرى من النظام.</t>
+  1. **حراسة الاختبارات (`test-guard`):** التحقق من أن الاختبارات تفحص سلوك النظام الفعلي ومنع Mocks الوهمية.
+  2. **قاعدة التغطية الإجبارية:** اختبار مسار النجاح، الفشل، والحالات الطرفية (Network Off, Lifecycle).</t>
         </is>
       </c>
     </row>
@@ -929,36 +918,34 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>11. خطاف إدارة النسخ والمستودعات</t>
+          <t>11. خطاف معالجة الأخطاء والأعطال</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
+          <t>حدث خطأ, التطبيق توقف, Crash</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Gemini 3.6 Flash (Medium)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager]</t>
+          <t>[debugger]</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
+          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من حالة المستودع:** فحص حالة Git باستخدام `git status` ومعرفة الملفات المعدلة والمحذوفة والجديدة.
-  2. **التنظيم والتصنيف:** مساعدة المطور في فرز الملفات، واستثناء الملفات غير الضرورية (تحديث `.gitignore`).
-  3. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وواضحة، وإنشاء فروع عند الحاجة (Branching)، وحل تعارضات الدمج، ثم دفع التغييرات إلى GitHub بأمان.</t>
+  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل وعزله وإصلاحه بأقل تعديل كافٍ.</t>
         </is>
       </c>
     </row>
@@ -968,37 +955,35 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>12. خطاف تحديث الإنجازات</t>
+          <t>12. خطاف إدارة النسخ والمستودعات</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
+          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+ البديل: `Gemini 3.6 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager], [docs-guard]</t>
+          <t>[git-github-manager]</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>صياغة التعديلات كإنجازات ومطابقتها برمجياً وتحديث README.md و hooks_user_guide.md ثم الرفع لـ GitHub.</t>
+          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs-vs-Code Drift).
-  3. **صياغة الإنجازات وتحديث التوثيق:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وتحديث ملف `README.md` وملف [`hooks_user_guide.md`](file:///f:/AI%20PROJECTS/Blind%20App/hooks_user_guide.md).
-  4. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديلات وإجراء الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
+  1. **التحقق من حالة المستودع:** فحص حالة Git واستثناء الملفات غير الضرورية في `.gitignore`.
+  2. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وحل التعارضات ودفع التغييرات إلى GitHub.</t>
         </is>
       </c>
     </row>
@@ -1008,38 +993,34 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>13. خطاف الذاكرة المستدامة</t>
+          <t>13. خطاف تحديث الإنجازات</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>حفظ ذاكرة, تحديث السياق, سجّل هذا</t>
+          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `GPT-OSS 120B (Medium)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>[persistent-memory-engine]</t>
+          <t>[git-github-manager], [docs-guard]</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>التقاط الدروس والقرارات وتخزينها في MEMORY_STORE.md وتصديرها للوكلاء.</t>
+          <t>صياغة التعديلات كإنجازات ومطابقتها برمجياً وتحديث README.md و hooks_user_guide.md ثم الرفع لـ GitHub.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فلترة وتدقيق الدروس (LESSON VALIDATION):** يُمنع تسجيل معلومات بديهية أو عامة. يجب أن تكون الذكريات مركزة على القواعد المعمارية الجديدة، حيل تقنية فريدة، أو تحذيرات من أخطاء مكررة. يجب تضمين قسم `[ANTI-PATTERN AVOIDED]` لكل درس لمنع تكرار الخطأ.
-  2. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية لاستخراج القرارات المعمارية العميقة والحلول.
-  3. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
-  4. **التصدير الانتقائي (Export):** تحديث حزمة السياق لكل وكيل حسب بروتوكول التصدير في `MEMORY_EXPORT_PROTOCOL.md`.
-  5. **التنقيح (Prune):** مراجعة الذكريات القديمة وحذف المتقادمة أو المتناقضة.</t>
+  1. **قراءة السجل ومطابقة التوثيق (`docs-guard`):** مراجعة التغييرات الأخيرة وصياغة الإنجازات وتحديث `README.md`.</t>
         </is>
       </c>
     </row>
@@ -1049,37 +1030,34 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>14. خطاف النجاح والتحليل البعدي</t>
+          <t>14. خطاف الذاكرة المستدامة</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>تم بنجاح, انتهى المشروع بنجاح</t>
+          <t>حفظ ذاكرة, تحديث السياق, سجّل هذا</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+ البديل: `GPT-OSS 120B (Medium)`</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>[agent-optimizer]</t>
+          <t>[persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
+          <t>التقاط الدروس والقرارات وتخزينها في MEMORY_STORE.md وتصديرها للوكلاء.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات التي واجهت الفريق والحلول البرمجية الفعالة التي تم تطبيقها.
-  2. **تحديث سجل التعلم (Learning Log):** توثيق المشاكل البرمجية المكتشفة وحلولها مباشرة في القسم الثامن من ملف `AGENTS.md` لتجنب تكرارها.
-  3. **تطوير مهارات الفريق:** مراجعة وتعديل مهارات الوكلاء وتحديث التعليمات تلقائياً.
-  4. **سد الفجوات البرمجية:** استدعاء الوكيل `[github-talent-scout]` للبحث عن أي مكتبات أو أدوات مفتوحة المصدر يمكنها تسريع العمل مستقبلاً ودمجها.</t>
+  1. **التقاط وتخزين الدروس:** حفظ القرارات المعمارية وتفضيلات المستخدم في `MEMORY_STORE.md`.</t>
         </is>
       </c>
     </row>
@@ -1089,36 +1067,34 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>15. خطاف تنظيم وترتيب الأجهزة الشامل</t>
+          <t>15. خطاف النجاح والتحليل البعدي</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>رتب جهازى, فرز الملفات, ترتيب ملفات</t>
+          <t>تم بنجاح, انتهى المشروع بنجاح</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Gemini 3.6 Flash (Medium)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>[windows-c-drive-optimizer], [windows-file-organizer]</t>
+          <t>[agent-optimizer]</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>ترتيب ملفات جذور الأقراص بالكامل مع تنظيف وتحسين مساحة قرص الـ C بآن واحد.</t>
+          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فرز وتصنيف جذور الأقراص:** نقل الملفات السائبة بالكامل لمجلدات مخصصة وآمنة.
-  2. **تنظيف وتحسين النظام:** تحفيز وكيل C لضغط النظام وتفريغ الفيديوهات المؤقتة لزيادة السرعة والمساحة معاً.
-  3. **فحص سلامة الروابط وتوليد الفهارس:** التحقق من Junction Links وتحديث الفهارس لـ NotebookLM.</t>
+  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات وتحديث سجل التعلم وسد الفجوات.</t>
         </is>
       </c>
     </row>
@@ -1128,36 +1104,34 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>16. خطاف ترتيب الملفات لمسار محدد</t>
+          <t>16. خطاف تنظيم وترتيب الأجهزة الشامل</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>رتب المسار, نظم المجلد, ترتيب مسار</t>
+          <t>رتب جهازى, فرز الملفات, ترتيب ملفات</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.6 Flash (Medium)` 
- البديل: `Gemini 3.5 Flash (Medium)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Gemini 3.6 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>[windows-file-organizer]</t>
+          <t>[windows-c-drive-optimizer], [windows-file-organizer]</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>تنظيم وفرز الملفات داخل مجلد أو مسار مخصص يحدده المستخدم بذكاء ودقة.</t>
+          <t>ترتيب ملفات جذور الأقراص بالكامل مع تنظيف وتحسين مساحة قرص الـ C بآن واحد.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تحديد وفحص المسار المستهدف:** التحقق من وجود المجلد المخصص وقراءة هيكل الملفات والمجلدات بداخله.
-  2. **تصنيف الملفات حسب النوع والتاريخ:** فرز الملفات حسب امتداداتها (مستندات، صور، فيديوهات، أكواد) أو تاريخ إنشائها.
-  3. **إعادة التسمية والتنظيم:** نقل الملفات إلى مجلدات فرعية مخصصة مع إعادة تسمية خالية من التعارضات.</t>
+  1. **فرز وتصنيف جذور الأقراص:** تنظيف وتحسين مساحة قرص C وترتيب الملفات السائبة.</t>
         </is>
       </c>
     </row>
@@ -1167,37 +1141,34 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>17. خطاف إدارة تليجرام</t>
+          <t>17. خطاف ترتيب الملفات لمسار محدد</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>شغل البوت, تفعيل تليجرام, Telegram Bot</t>
+          <t>رتب المسار, نظم المجلد, ترتيب مسار</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.5 Flash (Medium)` 
- البديل: `Gemini 3.1 Pro (Low)`</t>
+          <t>الأساسي: `Gemini 3.6 Flash (Medium)` 
+ البديل: `Gemini 3.5 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>[devops-deployer], [persistent-memory-engine]</t>
+          <t>[windows-file-organizer]</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>تشغيل بوت تليجرام في الخلفية بنمط الاستماع للطلبات عن بعد دون تعارض.</t>
+          <t>تنظيم وفرز الملفات داخل مجلد أو مسار مخصص يحدده المستخدم بذكاء ودقة.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من البيئة:** فحص وجود رمز البوت (TELEGRAM_BOT_TOKEN) والاعتماديات.
-  2. **معالجة التعارض (Conflict Resolution):** رصد وإنهاء أي عمليات بوت سابقة معلقة (معالجة خطأ 409 Conflict) عبر `taskkill`.
-  3. **التشغيل بنمط الاستماع الفردي:** تشغيل السكربت `poll_once.py` في الخلفية (One-Shot Polling) ليستمع لطلب واحد ويخرج، مما يوقظ الوكيل للعمل.
-  4. **إشعار الجاهزية:** تأكيد نجاح التشغيل واستعداد البوت لاستقبال الأوامر عبر التطبيق.</t>
+  1. **تنظيم وفرز الملفات:** تصنيف الملفات داخل مجلد محدد بذكاء ودقة.</t>
         </is>
       </c>
     </row>
@@ -1207,37 +1178,34 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>18. خطاف التدقيق البرمجي الشامل وحراسة الجودة</t>
+          <t>18. خطاف إدارة تليجرام</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
+          <t>شغل البوت, تفعيل تليجرام, Telegram Bot</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+          <t>الأساسي: `Gemini 3.5 Flash (Medium)` 
+ البديل: `Gemini 3.1 Pro (Low)`</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
+          <t>[devops-deployer], [persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
+          <t>تشغيل بوت تليجرام في الخلفية بنمط الاستماع للطلبات عن بعد دون تعارض.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود النظيف (`clean-code-guard`):** مراجعة جميع التغييرات البرمجية الأخيرة للتأكد من عدم ابتلاع الأخطاء، صغر حجم الدوال، غياب الكود المكرر، ودقة التسميات ومطابقة المعايير المعمارية.
-  2. **حراسة جودة الاختبارات (`test-guard`):** فحص جميع ملفات الاختبار للتحقق من عدم وجود Mocks وهمية أو اختبارات فارغة لا تكتشف الأخطاء الحقيقية.
-  3. **حراسة التوثيق ومطابقة الرموز (`docs-guard`):** مطابقة كافة ملفات التوثيق والـ Markdown مع الكود البرمجي الفعلي لضمان عدم وجود أي انحراف (Docs-vs-Code Drift).
-  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.</t>
+  1. **التشغيل بنمط الاستماع الفردي (One-Shot Polling):** تشغيل البوت للاستماع لطلب واحد دون تعارض مع بيئة التطوير.</t>
         </is>
       </c>
     </row>
@@ -1247,38 +1215,34 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>19. خطاف استكشاف وتكامل الموارد العالمية</t>
+          <t>19. خطاف التدقيق البرمجي الشامل وحراسة الجودة</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل hooks_user_guide.md ومزامنة المنظومة.</t>
+          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص وتقييم المورد (`resource-scout-integrator` + `github-talent-scout`):** استلام رابط المستودع الخارجي وفحص ملفات README والأكواد وتحديد ما إذا كان يُحدث نقلة نوعية واستبعاد ما لا يتوافق مع البيئة.
-  2. **بناء وهيكلة المهارات (`skill-forge-builder`):** استخراج المهارات الفعالة وصياغة ملفات `SKILL.md` وفق المعايير العالمية عبر `skill-creator` و `find-skills`.
-  3. **التعميم العالمي (`global-deployment`):** نشر المهارات في `C:\Users\Kt\.gemini\config\skills/` لتصبح متاحة لكل المشاريع.
-  4. **تحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل المستخدم (`agent-optimizer` + `frontend-design-builder`):** إضافة المهارات للخطافات ذات الصلة، وتحديث `hooks_user_guide.md` و `USER_GUIDE.md`، وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx` وتشغيل `update_html.py` لتحديث تطبيق مكتبة الأوامر التفاعلي (`03_Dynamic_Prompt_Library/index.html`).
-  5. **مزامنة المستودع العام سحابياً (`git-github-manager`):** تشغيل `sync_global_ecosystem.py` لمزامنة كامل منظومة الوكلاء والمهارات والدليل مع مستودع `Claude-Antigravity-Workspace` ورفعه إلى GitHub.</t>
+  1. **تفعيل بوابات الحماية الثلاث:** فحص الكود النظيف (`clean-code-guard`)، سلامة الاختبارات (`test-guard`)، ومطابقة التوثيق (`docs-guard`).</t>
         </is>
       </c>
     </row>
@@ -1288,38 +1252,226 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>20. خطاف المزامنة السحابية الشاملة ومطابقة المنظومة</t>
+          <t>20. خطاف استكشاف وتكامل الموارد العالمية</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>مزامنة المنظومة, مزامنة المستودع العام, تحديث المنظومة العالمية, sync ecosystem, sync workspace</t>
+          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>[resource-scout-integrator], [ui-ux-pro-max], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل hooks_user_guide.md ومزامنة المنظومة.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **استيراد وتعميم المهارات العالمية:** تحليل المستودعات الخارجية وبناء مهارات `SKILL.md` ونشرها عالمياً وتحديث المنظومة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>21. خطاف المزامنة السحابية والمساهمة المجتمعية</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>مزامنة المنظومة, sync ecosystem, ارسل pull request, مساهمة في المستودع, create PR, contribute repo</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.7 Flash (High)` 
  البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>[git-github-manager], [persistent-memory-engine], [agent-optimizer], [docs-guard]</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>مطابقة ومزامنة كافة الإضافات (Plugins)، المراجع والذاكرة، إعدادات MCP، المهارات والوكلاء، وتحديث الإكسيل ومكتبة الأوامر، ورفعها لـ GitHub بتطابق 100%.</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من سلامة المكونات والبيئة (`agent-optimizer`):** فحص حزم الإضافات (Plugins)، المهارات، والوكلاء والتكوينات العالمية في `~/.gemini/config/` ومقارنتها بالمشروع.
-  2. **تحديث ملفات الإكسيل وتطبيق مكتبة الأوامر:** تشغيل `convert_hooks_to_sheets.py` و `update_html.py` لتحديث `HOOKS_GUIDE.xlsx` و `index.html` بكافة الخطافات وتفاصيلها.
-  3. **تشغيل محرك المزامنة الشاملة (`sync_global_ecosystem.py`):** نسخ ومطابقة كافة الإضافات (Plugins)، والمراجع والذاكرة (References)، والمهارات، والوكلاء، وإعدادات MCP إلى `Claude-Antigravity-Workspace` بضمان تطابق 100%.
-  4. **فحص ومطابقة التوثيق (`docs-guard`):** مراجعة سلامة `README.md`, `USER_GUIDE.md`, `hooks_user_guide.md` لضمان عدم وجود أي انحراف.
-  5. **الالتزام والرفع التلقائي إلى GitHub (`git-github-manager`):** تنفيذ `git commit` موثق ودفع كافة التحديثات إلى المستودع العام [Claude-Antigravity-Workspace](https://github.com/ibrahimalkateb965-tech/Claude-Antigravity-Workspace) على GitHub بنقرة واحدة.
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>للمطور المالك: مطابقة ومزامنة كافة الإضافات والمهارات وتطبيق الأوامر مع GitHub. للمساهمين والمجتمع: تجهيز فرع الميزة وإنشاء وتوجيه Pull Request للمستودع المركزي للمشاركة.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **المسار الأول (للمطور المالك / Maintainer):**
+     - تشغيل `sync_global_ecosystem.py` لمطابقة كامل منظومة الوكلاء والمهارات والمراجع مع المسار العالمي ورفعها إلى مستودع GitHub الرئيسي بنقرة واحدة.
+  2. **المسار الثاني (للمساهمين والمجتمع / Community &amp; Contributors):**
+     - عند إضافة مهارة أو ميزة جديدة في نسخة Fork، يقوم الخطاف بفحص توافق الكود والتوثيق مع معايير Autovem.
+     - إنشاء فرع مساهمة (Feature Branch) وصياغة رسالة الالتزام وفق مواصفات Conventional Commits.
+     - فتح وتوجيه رابط **Pull Request** تلقائياً إلى المستودع المركزي [Claude-Antigravity-Workspace على GitHub](https://github.com/ibrahimalkateb965-tech/Claude-Antigravity-Workspace) لمراجعتها ودمجها لصالح المجتمع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>22. خطاف قيادة وإدارة الأسطول التشاركي</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>أسطول الـ CLIs, تشغيل الأسطول, تنسيق الأسطول, fleet orchestrator, multi cli fleet, إدارة الأسطول</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [code-architect], [agent-optimizer], [persistent-memory-engine]</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>تفعيل وضبط أسطول الوكلاء المتعدد، إدارة وتنسيق التكليف بين CLIs، حوكمة بوابات مراجعة الأكواد، وترشيد التوكنز.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **التهيئة والتوليد التلقائي (Auto-Provisioning):**
+     - فحص وجود مجلد `fleet_templates/` وملف `fleet_config.json` في المشروع وتوليدهما تلقائياً عند عدم وجودهما.
+  2. **توزيع المسؤوليات والحدود الحصرية وضبط النماذج:**
+     - تحديد ملكية الملفات والمهام في `fleet_config.json` لمنع التصادم:
+       - **Claude Code CLI** (النموذج: `Claude 5 Opus / Opus Max`): التخطيط والمراجعة المعمارية، **التنفيذ الحصري لكافة الاختبارات التلقائية**، واعتماد الأكواد وبوابات الجودة (Quality Gates).
+       - **OpenCode CLI** (النموذج: `Ox Alpha Unlimited`): التنفيذ الطرفي، إدارة قواعد البيانات Drift/ORM، وعملاء الاتصال والبيانات (كتابة وبناء فقط دون تشغيل أي اختبارات).
+       - **Antigravity IDE** (النموذج: `Gemini 3.7 Flash High`): بناء الواجهات والـ Domain Logic، إدارة الذاكرة المستدامة، وهندسة السياق (كتابة وبناء فقط دون تشغيل أي اختبارات).
+  3. **التشغيل المباشر لأدوات الـ CLI (Headless Direct Invocation):**
+     - تشغيل واستدعاء أدوات الـ CLI المثبتة مباشرة عبر سطر الأوامر غير التفاعلي:
+       - استدعاء `Claude Code CLI` للمراجعة المعمارية وتشغيل الاختبارات وتدقيق الكود عبر: `claude -p "&lt;prompt&gt;"` أو `claude --print`.
+       - استدعاء `OpenCode CLI` لتنفيذ الأوامر السريعة والطرفية وبناء قواعد البيانات عبر: `opencode run "&lt;message&gt;"`.
+     - معالجة وإدراج مخرجات الـ CLIs تلقائياً في دورة التطوير وبوابات الجودة.
+  4. **التحويل المستدام لنمط المحادثة (Session-Wide Fleet Mode Transformation):**
+     - **قاعدة حاسمة:** بمجرد استدعاء وتفعيل الخطاف 22 (بالمحفزات المعتمدة أو ذكر خطاف 22)، يدخل المساعد فوراً ومستداماً في **نمط قيادة الأسطول (Fleet Command Mode)** لكامل ما تبقى من الجلسة.
+     - تتحول كافة طلبات وأوامر المستخدم اللاحقة تلقائياً إلى أوامر وهياكل تفويض وتنسيق موجهة للأسطول باللغة الإنجليزية وفق الهيكل المعياري المعتمد (`Template 02: Task Delegation Protocol` و `Template 03: Code Review Audit`) مع حصر الملكية الدليلية، وفرض حظر تشغيل الاختبارات على غير Claude Code، وتأكيد خلو الأخطاء (`flutter analyze = 0`) دون الحاجة لتكرار تفعيل الخطاف في كل رسالة.
+  5. **احتكار الفحص والاختبار لـ Claude Code فقط (Testing Monopoly):**
+     - يُحظر حظراً تاماً تشغيل الاختبارات بواسطة OpenCode أو Antigravity. يتولى Claude Code تشغيل الاختبارات وفحص واعتماد أي كود مكتوب قبل دمجه.
+  6. **حوكمة بوابات الجودة وترشيد التوكنز:**
+     - مراجعة diffs كل مرحلة وفرض اللغة الإنجليزية بالكامل في طرفيات الـ CLIs مع حظر كتابة البويلربليت على النماذج العليا.
+  7. **إدارة الكوتا والتسليم السلس (Quota Failover &amp; Re-entry):**
+      - ضمان استمرارية المشروع وتسليم القيادة بسلاسة عند امتلاء كوتا أي نموذج مع تطبيق بروتوكول إعادة الدخول عند تجدد الحصة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>23. خطاف تحويل وأتمتة سكربتات المشاريع إلى MCP</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>حول إلى MCP, تحويل سكربتات لـ MCP, بناء أدوات MCP, convert scripts to mcp, scripts to mcp, ترقية السكربتات</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>[mcp-tool-builder], [script-to-mcp-converter], [code-architect], [agent-optimizer]</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>مسح سكربتات بايثون المبعثرة في مسار المشروع، تجريد منطق العمل وبناء دوال FastMCP ونماذج Pydantic، تسجيل الخادم، وأرشفة السكربتات في القرص الثانوي (G:) وحماية قرص C:.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **المسح والاكتشاف الشامل (Script Discovery &amp; AST Analysis):**
+     - تشغيل `project_scripts_to_mcp.py` لمسح كافة ملفات بايثون المتناثرة داخل مجلدات المشروع، وتحليل أسماء الدوال، المعاملات، والمخرجات برمجياً.
+  2. **تجريد المنطق وهيكلة Pydantic (Decoupling &amp; Schema Generation):**
+     - فصل كود المعالجة عن المسارات الصلبة (Hardcoded Paths)، وصياغة كلاسات Pydantic Request لكل أداة لضمان التحقق من صحة المدخلات.
+  3. **البناء والتسجيل في FastMCP (FastMCP Tool Registration):**
+     - دمج الدوال في خادم FastMCP موحد ومستقر مع إلزام ترميز UTF-8 ودعم التزامن `asyncio.to_thread`.
+     - تسجيل الخادم وأدواته في `mcp_config.json` للـ IDE والوكلاء.
+  4. **الأرشفة الآمنة وحماية قرص النظام (Secondary Drive Archiving):**
+     - نقل السكربتات القديمة تلقائياً إلى مجلد أرشيف منظم على القرص الثانوي (`G:\_scripts_archive` أو حسب القرص المخصص) مع حظر الحفظ على قرص النظام `C:\`.
+  5. **تحديث مهارات الوكلاء والذاكرة:**
+     - تحديث بطاقات المهارات في `.agents/skills` لتمكين الوكلاء المتخصصين من استدعاء أدوات الـ MCP الجديدة مباشرة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>24. خطاف أتمتة مسارات العمل ووكلاء n8n الذكية</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ابني مسار n8n, أتمتة n8n, وكيل n8n, n8n ai agent, n8n workflow, تصميم ورك فلو</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>[n8n-ai-agent-architect], [mcp-tool-builder], [backend-architect], [agent-optimizer]</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>تصميم وبناء مسارات عمل ذكية مؤتمتة على n8n، ربط الوكلاء المتعددين (Multi-Agent Sub-workflows)، تتبع التحويلات وتأهيل العملاء، وربط خوادم MCP وقواعد البيانات الموجهة بالذكاء الاصطناعي.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **التصميم المعماري للمسار (`n8n-ai-agent-architect`):**
+     - اختيار النمط المعماري المناسب (Multi-Agent Router, ReAct Tools Agent, Evaluator-Optimizer Loop, أو Human-in-the-Loop).
+  2. **بناء وهيكلة أدوات الاستدعاء (Tool Calling &amp; JSON Schemas):**
+     - بناء وتوثيق أدوات HTTP Request و Custom JavaScript Tools مع فرض JSON Schema صارم يمنع هلوسة المعاملات.
+  3. **إدارة طبقات الذاكرة (Short-Term &amp; Vector Memory):**
+     - ربط الذاكرة القصيرة (Window Buffer) والذاكرة المستمرة (Postgres/Redis) ومخازن المتجهات الدلالية (Qdrant/Pinecone/Supabase).
+  4. **أتمتة العمليات التسويقية وتأهيل العملاء (Marketing &amp; CRM Pipelines):**
+     - بناء مسارات استقبال وتحليل بيانات العملاء المحتملين من Google Ads و Facebook وتوجيه الإشعارات اللحظية عبر WhatsApp و Slack وتحديث الـ CRM.
+  5. **تحصين الانقطاع ومعالجة الأخطاء (Fault Tolerance &amp; Sub-workflow Retries):**
+     - إضافة مسارات الخطأ (Error Trigger) وإعادة المحاولة مع التراجع التلقائي (Exponential Backoff) ونماذج LLM البديلة.
 &lt;/div&gt;</t>
         </is>
       </c>
@@ -1390,37 +1542,35 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>9. خطاف الفحص والاختبار التلقائي</t>
+          <t>9. خطاف مراجعة وتحديث المكتبات والنماذج</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>قم بالاختبار, جاهز للتجربة</t>
+          <t>تحديث الاعتماديات, تحديث المكتبات, تحديث النماذج, معايرة النماذج, update models</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Gemini 3.6 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[android-testing], [test-guard], [code-reviewer-quality]</t>
+          <t>[github-talent-scout], [code-architect], [agent-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تشغيل اختبارات الوحدة وفحص جودة الكود واختبار السلوك الفعلي بدون Mock مفرط.</t>
+          <t>فحص ملفات Gradle وتحديث المكتبات، والتحقق التلقائي عبر الإنترنت (antigravity.google) لتحديث مصفوفة النماذج ودليل hooks_user_guide.md دون لقطات شاشة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التقمص (Persona):** يتصرف الوكيل كمدير فحص جودة صارم (Pre-Flight Inspector &amp; Senior DevOps QA). بصرامة تامة وبدون أي مجاملات.
-  2. **حراسة الاختبارات (`test-guard`):** التحقق من أن الاختبارات تفحص سلوك النظام الفعلي ومخرجاته القابلة للملاحظة، ومنع الاختبارات الوهمية (Tautological Tests) والـ Mocks الزائدة.
-  3. **قاعدة التغطية الإجبارية (TEST COVERAGE MANDATE):** يُرفض أي اختبار يغطي مسار النجاح فقط (Happy Path). يجب كتابة اختبار للنجاح، الفشل، والحالات الطرفية (مثل: Network Off، Configuration Change).
-  4. **تقرير الفحص الصارم:** تزويد المطور بتقرير يحاكي المطالبة القياسية: `[BLOCKERS]`, `[WARNINGS]`, `[PRE-FLIGHT FIXES]`, `[GO / NO-GO]`.</t>
+  1. **فحص إصدارات المكتبات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
+  2. **الاستكشاف والمعايرة التلقائية للنماذج عبر الإنترنت (Online Model Discovery):** الاستعلام الفوري عبر المصادر الرسمية (antigravity.google, docs.anthropic.com) ومعايرة مصفوفة النماذج.</t>
         </is>
       </c>
     </row>
@@ -1490,12 +1640,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>10. خطاف معالجة الأخطاء والأعطال</t>
+          <t>10. خطاف الفحص والاختبار التلقائي</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>حدث خطأ, التطبيق توقف, Crash</t>
+          <t>قم بالاختبار, جاهز للتجربة</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1506,20 +1656,19 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[debugger]</t>
+          <t>[android-testing], [test-guard], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
+          <t>تشغيل اختبارات الوحدة وفحص جودة الكود واختبار السلوك الفعلي بدون Mock مفرط.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل.
-  2. **عزل المشكلة:** حصر الكود المسبب للأخطاء لمعرفة إن كان يتعلق بالشبكة، قاعدة البيانات، أو دورة حياة المكونات.
-  3. **اقتراح وتثبيت الحل:** تطبيق التعديل الأدنى الكافي لحل المشكلة مع حماية الأجزاء الأخرى من النظام.</t>
+  1. **حراسة الاختبارات (`test-guard`):** التحقق من أن الاختبارات تفحص سلوك النظام الفعلي ومنع Mocks الوهمية.
+  2. **قاعدة التغطية الإجبارية:** اختبار مسار النجاح، الفشل، والحالات الطرفية (Network Off, Lifecycle).</t>
         </is>
       </c>
     </row>
@@ -1589,36 +1738,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>11. خطاف إدارة النسخ والمستودعات</t>
+          <t>11. خطاف معالجة الأخطاء والأعطال</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
+          <t>حدث خطأ, التطبيق توقف, Crash</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Gemini 3.6 Flash (Medium)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager]</t>
+          <t>[debugger]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
+          <t>تحليل سجلات الأخطاء والـ Stack Trace وعزل الكود المسبب للمشكلة وإصلاحه.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من حالة المستودع:** فحص حالة Git باستخدام `git status` ومعرفة الملفات المعدلة والمحذوفة والجديدة.
-  2. **التنظيم والتصنيف:** مساعدة المطور في فرز الملفات، واستثناء الملفات غير الضرورية (تحديث `.gitignore`).
-  3. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وواضحة، وإنشاء فروع عند الحاجة (Branching)، وحل تعارضات الدمج، ثم دفع التغييرات إلى GitHub بأمان.</t>
+  1. **تحليل الـ Stack Trace:** قراءة السجلات بدقة وتحديد السطر المسبب للخلل وعزله وإصلاحه بأقل تعديل كافٍ.</t>
         </is>
       </c>
     </row>
@@ -1688,37 +1835,35 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>12. خطاف تحديث الإنجازات</t>
+          <t>12. خطاف إدارة النسخ والمستودعات</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
+          <t>نظم جيت, ارفع لجيتهاب, تحديث المستودع, git commit</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+ البديل: `Gemini 3.6 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[git-github-manager], [docs-guard]</t>
+          <t>[git-github-manager]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>صياغة التعديلات كإنجازات ومطابقتها برمجياً وتحديث README.md و hooks_user_guide.md ثم الرفع لـ GitHub.</t>
+          <t>تهيئة المشاريع الجديدة على Git، إدارة التفرعات، وحل تعارضات الدمج ورفعها لـ GitHub بشكل نظيف.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة السجل والذاكرة:** مراجعة التغييرات الأخيرة في الملفات وقراءة `MEMORY_STORE.md` لاستخلاص ما تم إنجازه.
-  2. **مطابقة التوثيق (`docs-guard`):** مطابقة كل رمز برمجي أو مسار أو دالة مذكورة في التوثيق مع الكود الحقيقي لمنع أي تباين أو اختلاق (Docs-vs-Code Drift).
-  3. **صياغة الإنجازات وتحديث التوثيق:** كتابة الإنجازات بنسق احترافي كنقاط موجزة، وتحديث ملف `README.md` وملف [`hooks_user_guide.md`](file:///f:/AI%20PROJECTS/Blind%20App/hooks_user_guide.md).
-  4. **الرفع التلقائي (Commit &amp; Push):** إضافة التعديلات وإجراء الحفظ، ثم الرفع التلقائي إلى GitHub مباشرة كخطوة نهائية متصلة.</t>
+  1. **التحقق من حالة المستودع:** فحص حالة Git واستثناء الملفات غير الضرورية في `.gitignore`.
+  2. **التنفيذ والرفع:** كتابة رسائل Commit احترافية وحل التعارضات ودفع التغييرات إلى GitHub.</t>
         </is>
       </c>
     </row>
@@ -1788,38 +1933,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>13. خطاف الذاكرة المستدامة</t>
+          <t>13. خطاف تحديث الإنجازات</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>حفظ ذاكرة, تحديث السياق, سجّل هذا</t>
+          <t>حدث الإنجازات, تحديث README, وثق الإنجازات</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `GPT-OSS 120B (Medium)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[persistent-memory-engine]</t>
+          <t>[git-github-manager], [docs-guard]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>التقاط الدروس والقرارات وتخزينها في MEMORY_STORE.md وتصديرها للوكلاء.</t>
+          <t>صياغة التعديلات كإنجازات ومطابقتها برمجياً وتحديث README.md و hooks_user_guide.md ثم الرفع لـ GitHub.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فلترة وتدقيق الدروس (LESSON VALIDATION):** يُمنع تسجيل معلومات بديهية أو عامة. يجب أن تكون الذكريات مركزة على القواعد المعمارية الجديدة، حيل تقنية فريدة، أو تحذيرات من أخطاء مكررة. يجب تضمين قسم `[ANTI-PATTERN AVOIDED]` لكل درس لمنع تكرار الخطأ.
-  2. **التقاط السياق (Capture):** يقوم الوكيل `[persistent-memory-engine]` بتحليل الجلسة الحالية لاستخراج القرارات المعمارية العميقة والحلول.
-  3. **التخزين الهيكلي (Store):** كتابة الذكريات المستخرجة في `MEMORY_STORE.md` بصيغة YAML الموحدة مع التصنيف بالوسوم والتوقيت.
-  4. **التصدير الانتقائي (Export):** تحديث حزمة السياق لكل وكيل حسب بروتوكول التصدير في `MEMORY_EXPORT_PROTOCOL.md`.
-  5. **التنقيح (Prune):** مراجعة الذكريات القديمة وحذف المتقادمة أو المتناقضة.</t>
+  1. **قراءة السجل ومطابقة التوثيق (`docs-guard`):** مراجعة التغييرات الأخيرة وصياغة الإنجازات وتحديث `README.md`.</t>
         </is>
       </c>
     </row>
@@ -1889,37 +2030,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>14. خطاف النجاح والتحليل البعدي</t>
+          <t>14. خطاف الذاكرة المستدامة</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تم بنجاح, انتهى المشروع بنجاح</t>
+          <t>حفظ ذاكرة, تحديث السياق, سجّل هذا</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+ البديل: `GPT-OSS 120B (Medium)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[agent-optimizer]</t>
+          <t>[persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
+          <t>التقاط الدروس والقرارات وتخزينها في MEMORY_STORE.md وتصديرها للوكلاء.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات التي واجهت الفريق والحلول البرمجية الفعالة التي تم تطبيقها.
-  2. **تحديث سجل التعلم (Learning Log):** توثيق المشاكل البرمجية المكتشفة وحلولها مباشرة في القسم الثامن من ملف `AGENTS.md` لتجنب تكرارها.
-  3. **تطوير مهارات الفريق:** مراجعة وتعديل مهارات الوكلاء وتحديث التعليمات تلقائياً.
-  4. **سد الفجوات البرمجية:** استدعاء الوكيل `[github-talent-scout]` للبحث عن أي مكتبات أو أدوات مفتوحة المصدر يمكنها تسريع العمل مستقبلاً ودمجها.</t>
+  1. **التقاط وتخزين الدروس:** حفظ القرارات المعمارية وتفضيلات المستخدم في `MEMORY_STORE.md`.</t>
         </is>
       </c>
     </row>
@@ -1989,36 +2127,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>15. خطاف تنظيم وترتيب الأجهزة الشامل</t>
+          <t>15. خطاف النجاح والتحليل البعدي</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>رتب جهازى, فرز الملفات, ترتيب ملفات</t>
+          <t>تم بنجاح, انتهى المشروع بنجاح</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Gemini 3.6 Flash (Medium)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[windows-c-drive-optimizer], [windows-file-organizer]</t>
+          <t>[agent-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>ترتيب ملفات جذور الأقراص بالكامل مع تنظيف وتحسين مساحة قرص الـ C بآن واحد.</t>
+          <t>إجراء تحليل بعدي للمشروع وتحديث سجل التعلم وسد الثغرات البرمجية.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فرز وتصنيف جذور الأقراص:** نقل الملفات السائبة بالكامل لمجلدات مخصصة وآمنة.
-  2. **تنظيف وتحسين النظام:** تحفيز وكيل C لضغط النظام وتفريغ الفيديوهات المؤقتة لزيادة السرعة والمساحة معاً.
-  3. **فحص سلامة الروابط وتوليد الفهارس:** التحقق من Junction Links وتحديث الفهارس لـ NotebookLM.</t>
+  1. **التحليل البعدي (Post-Mortem Analysis):** دراسة سجل المحادثة واستخراج العقبات وتحديث سجل التعلم وسد الفجوات.</t>
         </is>
       </c>
     </row>
@@ -2088,36 +2224,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>16. خطاف ترتيب الملفات لمسار محدد</t>
+          <t>16. خطاف تنظيم وترتيب الأجهزة الشامل</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>رتب المسار, نظم المجلد, ترتيب مسار</t>
+          <t>رتب جهازى, فرز الملفات, ترتيب ملفات</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.6 Flash (Medium)` 
- البديل: `Gemini 3.5 Flash (Medium)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Gemini 3.6 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[windows-file-organizer]</t>
+          <t>[windows-c-drive-optimizer], [windows-file-organizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تنظيم وفرز الملفات داخل مجلد أو مسار مخصص يحدده المستخدم بذكاء ودقة.</t>
+          <t>ترتيب ملفات جذور الأقراص بالكامل مع تنظيف وتحسين مساحة قرص الـ C بآن واحد.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **تحديد وفحص المسار المستهدف:** التحقق من وجود المجلد المخصص وقراءة هيكل الملفات والمجلدات بداخله.
-  2. **تصنيف الملفات حسب النوع والتاريخ:** فرز الملفات حسب امتداداتها (مستندات، صور، فيديوهات، أكواد) أو تاريخ إنشائها.
-  3. **إعادة التسمية والتنظيم:** نقل الملفات إلى مجلدات فرعية مخصصة مع إعادة تسمية خالية من التعارضات.</t>
+  1. **فرز وتصنيف جذور الأقراص:** تنظيف وتحسين مساحة قرص C وترتيب الملفات السائبة.</t>
         </is>
       </c>
     </row>
@@ -2187,37 +2321,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>17. خطاف إدارة تليجرام</t>
+          <t>17. خطاف ترتيب الملفات لمسار محدد</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>شغل البوت, تفعيل تليجرام, Telegram Bot</t>
+          <t>رتب المسار, نظم المجلد, ترتيب مسار</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.5 Flash (Medium)` 
- البديل: `Gemini 3.1 Pro (Low)`</t>
+          <t>الأساسي: `Gemini 3.6 Flash (Medium)` 
+ البديل: `Gemini 3.5 Flash (Medium)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[devops-deployer], [persistent-memory-engine]</t>
+          <t>[windows-file-organizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تشغيل بوت تليجرام في الخلفية بنمط الاستماع للطلبات عن بعد دون تعارض.</t>
+          <t>تنظيم وفرز الملفات داخل مجلد أو مسار مخصص يحدده المستخدم بذكاء ودقة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من البيئة:** فحص وجود رمز البوت (TELEGRAM_BOT_TOKEN) والاعتماديات.
-  2. **معالجة التعارض (Conflict Resolution):** رصد وإنهاء أي عمليات بوت سابقة معلقة (معالجة خطأ 409 Conflict) عبر `taskkill`.
-  3. **التشغيل بنمط الاستماع الفردي:** تشغيل السكربت `poll_once.py` في الخلفية (One-Shot Polling) ليستمع لطلب واحد ويخرج، مما يوقظ الوكيل للعمل.
-  4. **إشعار الجاهزية:** تأكيد نجاح التشغيل واستعداد البوت لاستقبال الأوامر عبر التطبيق.</t>
+  1. **تنظيم وفرز الملفات:** تصنيف الملفات داخل مجلد محدد بذكاء ودقة.</t>
         </is>
       </c>
     </row>
@@ -2287,37 +2418,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>18. خطاف التدقيق البرمجي الشامل وحراسة الجودة</t>
+          <t>18. خطاف إدارة تليجرام</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
+          <t>شغل البوت, تفعيل تليجرام, Telegram Bot</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+          <t>الأساسي: `Gemini 3.5 Flash (Medium)` 
+ البديل: `Gemini 3.1 Pro (Low)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
+          <t>[devops-deployer], [persistent-memory-engine]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
+          <t>تشغيل بوت تليجرام في الخلفية بنمط الاستماع للطلبات عن بعد دون تعارض.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود النظيف (`clean-code-guard`):** مراجعة جميع التغييرات البرمجية الأخيرة للتأكد من عدم ابتلاع الأخطاء، صغر حجم الدوال، غياب الكود المكرر، ودقة التسميات ومطابقة المعايير المعمارية.
-  2. **حراسة جودة الاختبارات (`test-guard`):** فحص جميع ملفات الاختبار للتحقق من عدم وجود Mocks وهمية أو اختبارات فارغة لا تكتشف الأخطاء الحقيقية.
-  3. **حراسة التوثيق ومطابقة الرموز (`docs-guard`):** مطابقة كافة ملفات التوثيق والـ Markdown مع الكود البرمجي الفعلي لضمان عدم وجود أي انحراف (Docs-vs-Code Drift).
-  4. **إصدار تقرير الجودة والحراسة:** تزويد المطور بتقرير شامل يحدد المخالفات المكتشفة وتصحيحاتها الفورية قبل الرفع والدمج.</t>
+  1. **التشغيل بنمط الاستماع الفردي (One-Shot Polling):** تشغيل البوت للاستماع لطلب واحد دون تعارض مع بيئة التطوير.</t>
         </is>
       </c>
     </row>
@@ -2486,38 +2614,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>19. خطاف استكشاف وتكامل الموارد العالمية</t>
+          <t>19. خطاف التدقيق البرمجي الشامل وحراسة الجودة</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
+          <t>تدقيق الجودة, فحص الكود النظيف, حراسة الجودة, clean code audit</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[resource-scout-integrator], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [test-guard], [docs-guard]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل hooks_user_guide.md ومزامنة المنظومة.</t>
+          <t>تفعيل بوابات الحماية الثلاث لفحص الكود النظيف، سلامة الاختبارات، ومطابقة التوثيق.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص وتقييم المورد (`resource-scout-integrator` + `github-talent-scout`):** استلام رابط المستودع الخارجي وفحص ملفات README والأكواد وتحديد ما إذا كان يُحدث نقلة نوعية واستبعاد ما لا يتوافق مع البيئة.
-  2. **بناء وهيكلة المهارات (`skill-forge-builder`):** استخراج المهارات الفعالة وصياغة ملفات `SKILL.md` وفق المعايير العالمية عبر `skill-creator` و `find-skills`.
-  3. **التعميم العالمي (`global-deployment`):** نشر المهارات في `C:\Users\Kt\.gemini\config\skills/` لتصبح متاحة لكل المشاريع.
-  4. **تحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل المستخدم (`agent-optimizer` + `frontend-design-builder`):** إضافة المهارات للخطافات ذات الصلة، وتحديث `hooks_user_guide.md` و `USER_GUIDE.md`، وتشغيل سكربت `convert_hooks_to_sheets.py` لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx` وتشغيل `update_html.py` لتحديث تطبيق مكتبة الأوامر التفاعلي (`03_Dynamic_Prompt_Library/index.html`).
-  5. **مزامنة المستودع العام سحابياً (`git-github-manager`):** تشغيل `sync_global_ecosystem.py` لمزامنة كامل منظومة الوكلاء والمهارات والدليل مع مستودع `Claude-Antigravity-Workspace` ورفعه إلى GitHub.</t>
+  1. **تفعيل بوابات الحماية الثلاث:** فحص الكود النظيف (`clean-code-guard`)، سلامة الاختبارات (`test-guard`)، ومطابقة التوثيق (`docs-guard`).</t>
         </is>
       </c>
     </row>
@@ -2587,12 +2711,109 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>20. خطاف المزامنة السحابية الشاملة ومطابقة المنظومة</t>
+          <t>20. خطاف استكشاف وتكامل الموارد العالمية</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>مزامنة المنظومة, مزامنة المستودع العام, تحديث المنظومة العالمية, sync ecosystem, sync workspace</t>
+          <t>استكشف المورد, حلل المستودع, تكامل المورد, scout resource, integrate repo</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[resource-scout-integrator], [ui-ux-pro-max], [github-talent-scout], [skill-forge-builder], [agent-optimizer], [frontend-design-builder], [git-github-manager]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>تحليل المستودعات الخارجية واستيراد المهارات وتعميمها وتحديث الخطافات والإكسيل وتطبيق مكتبة الأوامر ودليل hooks_user_guide.md ومزامنة المنظومة.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **استيراد وتعميم المهارات العالمية:** تحليل المستودعات الخارجية وبناء مهارات `SKILL.md` ونشرها عالمياً وتحديث المنظومة.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>21. خطاف المزامنة السحابية والمساهمة المجتمعية</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>مزامنة المنظومة, sync ecosystem, ارسل pull request, مساهمة في المستودع, create PR, contribute repo</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2608,17 +2829,348 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>مطابقة ومزامنة كافة الإضافات (Plugins)، المراجع والذاكرة، إعدادات MCP، المهارات والوكلاء، وتحديث الإكسيل ومكتبة الأوامر، ورفعها لـ GitHub بتطابق 100%.</t>
+          <t>للمطور المالك: مطابقة ومزامنة كافة الإضافات والمهارات وتطبيق الأوامر مع GitHub. للمساهمين والمجتمع: تجهيز فرع الميزة وإنشاء وتوجيه Pull Request للمستودع المركزي للمشاركة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **التحقق من سلامة المكونات والبيئة (`agent-optimizer`):** فحص حزم الإضافات (Plugins)، المهارات، والوكلاء والتكوينات العالمية في `~/.gemini/config/` ومقارنتها بالمشروع.
-  2. **تحديث ملفات الإكسيل وتطبيق مكتبة الأوامر:** تشغيل `convert_hooks_to_sheets.py` و `update_html.py` لتحديث `HOOKS_GUIDE.xlsx` و `index.html` بكافة الخطافات وتفاصيلها.
-  3. **تشغيل محرك المزامنة الشاملة (`sync_global_ecosystem.py`):** نسخ ومطابقة كافة الإضافات (Plugins)، والمراجع والذاكرة (References)، والمهارات، والوكلاء، وإعدادات MCP إلى `Claude-Antigravity-Workspace` بضمان تطابق 100%.
-  4. **فحص ومطابقة التوثيق (`docs-guard`):** مراجعة سلامة `README.md`, `USER_GUIDE.md`, `hooks_user_guide.md` لضمان عدم وجود أي انحراف.
-  5. **الالتزام والرفع التلقائي إلى GitHub (`git-github-manager`):** تنفيذ `git commit` موثق ودفع كافة التحديثات إلى المستودع العام [Claude-Antigravity-Workspace](https://github.com/ibrahimalkateb965-tech/Claude-Antigravity-Workspace) على GitHub بنقرة واحدة.
+  1. **المسار الأول (للمطور المالك / Maintainer):**
+     - تشغيل `sync_global_ecosystem.py` لمطابقة كامل منظومة الوكلاء والمهارات والمراجع مع المسار العالمي ورفعها إلى مستودع GitHub الرئيسي بنقرة واحدة.
+  2. **المسار الثاني (للمساهمين والمجتمع / Community &amp; Contributors):**
+     - عند إضافة مهارة أو ميزة جديدة في نسخة Fork، يقوم الخطاف بفحص توافق الكود والتوثيق مع معايير Autovem.
+     - إنشاء فرع مساهمة (Feature Branch) وصياغة رسالة الالتزام وفق مواصفات Conventional Commits.
+     - فتح وتوجيه رابط **Pull Request** تلقائياً إلى المستودع المركزي [Claude-Antigravity-Workspace على GitHub](https://github.com/ibrahimalkateb965-tech/Claude-Antigravity-Workspace) لمراجعتها ودمجها لصالح المجتمع.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>22. خطاف قيادة وإدارة الأسطول التشاركي</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>أسطول الـ CLIs, تشغيل الأسطول, تنسيق الأسطول, fleet orchestrator, multi cli fleet, إدارة الأسطول</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Opus 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[fleet-orchestrator], [code-architect], [agent-optimizer], [persistent-memory-engine]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>تفعيل وضبط أسطول الوكلاء المتعدد، إدارة وتنسيق التكليف بين CLIs، حوكمة بوابات مراجعة الأكواد، وترشيد التوكنز.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **التهيئة والتوليد التلقائي (Auto-Provisioning):**
+     - فحص وجود مجلد `fleet_templates/` وملف `fleet_config.json` في المشروع وتوليدهما تلقائياً عند عدم وجودهما.
+  2. **توزيع المسؤوليات والحدود الحصرية وضبط النماذج:**
+     - تحديد ملكية الملفات والمهام في `fleet_config.json` لمنع التصادم:
+       - **Claude Code CLI** (النموذج: `Claude 5 Opus / Opus Max`): التخطيط والمراجعة المعمارية، **التنفيذ الحصري لكافة الاختبارات التلقائية**، واعتماد الأكواد وبوابات الجودة (Quality Gates).
+       - **OpenCode CLI** (النموذج: `Ox Alpha Unlimited`): التنفيذ الطرفي، إدارة قواعد البيانات Drift/ORM، وعملاء الاتصال والبيانات (كتابة وبناء فقط دون تشغيل أي اختبارات).
+       - **Antigravity IDE** (النموذج: `Gemini 3.7 Flash High`): بناء الواجهات والـ Domain Logic، إدارة الذاكرة المستدامة، وهندسة السياق (كتابة وبناء فقط دون تشغيل أي اختبارات).
+  3. **التشغيل المباشر لأدوات الـ CLI (Headless Direct Invocation):**
+     - تشغيل واستدعاء أدوات الـ CLI المثبتة مباشرة عبر سطر الأوامر غير التفاعلي:
+       - استدعاء `Claude Code CLI` للمراجعة المعمارية وتشغيل الاختبارات وتدقيق الكود عبر: `claude -p "&lt;prompt&gt;"` أو `claude --print`.
+       - استدعاء `OpenCode CLI` لتنفيذ الأوامر السريعة والطرفية وبناء قواعد البيانات عبر: `opencode run "&lt;message&gt;"`.
+     - معالجة وإدراج مخرجات الـ CLIs تلقائياً في دورة التطوير وبوابات الجودة.
+  4. **التحويل المستدام لنمط المحادثة (Session-Wide Fleet Mode Transformation):**
+     - **قاعدة حاسمة:** بمجرد استدعاء وتفعيل الخطاف 22 (بالمحفزات المعتمدة أو ذكر خطاف 22)، يدخل المساعد فوراً ومستداماً في **نمط قيادة الأسطول (Fleet Command Mode)** لكامل ما تبقى من الجلسة.
+     - تتحول كافة طلبات وأوامر المستخدم اللاحقة تلقائياً إلى أوامر وهياكل تفويض وتنسيق موجهة للأسطول باللغة الإنجليزية وفق الهيكل المعياري المعتمد (`Template 02: Task Delegation Protocol` و `Template 03: Code Review Audit`) مع حصر الملكية الدليلية، وفرض حظر تشغيل الاختبارات على غير Claude Code، وتأكيد خلو الأخطاء (`flutter analyze = 0`) دون الحاجة لتكرار تفعيل الخطاف في كل رسالة.
+  5. **احتكار الفحص والاختبار لـ Claude Code فقط (Testing Monopoly):**
+     - يُحظر حظراً تاماً تشغيل الاختبارات بواسطة OpenCode أو Antigravity. يتولى Claude Code تشغيل الاختبارات وفحص واعتماد أي كود مكتوب قبل دمجه.
+  6. **حوكمة بوابات الجودة وترشيد التوكنز:**
+     - مراجعة diffs كل مرحلة وفرض اللغة الإنجليزية بالكامل في طرفيات الـ CLIs مع حظر كتابة البويلربليت على النماذج العليا.
+  7. **إدارة الكوتا والتسليم السلس (Quota Failover &amp; Re-entry):**
+      - ضمان استمرارية المشروع وتسليم القيادة بسلاسة عند امتلاء كوتا أي نموذج مع تطبيق بروتوكول إعادة الدخول عند تجدد الحصة.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>23. خطاف تحويل وأتمتة سكربتات المشاريع إلى MCP</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>حول إلى MCP, تحويل سكربتات لـ MCP, بناء أدوات MCP, convert scripts to mcp, scripts to mcp, ترقية السكربتات</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[mcp-tool-builder], [script-to-mcp-converter], [code-architect], [agent-optimizer]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>مسح سكربتات بايثون المبعثرة في مسار المشروع، تجريد منطق العمل وبناء دوال FastMCP ونماذج Pydantic، تسجيل الخادم، وأرشفة السكربتات في القرص الثانوي (G:) وحماية قرص C:.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **المسح والاكتشاف الشامل (Script Discovery &amp; AST Analysis):**
+     - تشغيل `project_scripts_to_mcp.py` لمسح كافة ملفات بايثون المتناثرة داخل مجلدات المشروع، وتحليل أسماء الدوال، المعاملات، والمخرجات برمجياً.
+  2. **تجريد المنطق وهيكلة Pydantic (Decoupling &amp; Schema Generation):**
+     - فصل كود المعالجة عن المسارات الصلبة (Hardcoded Paths)، وصياغة كلاسات Pydantic Request لكل أداة لضمان التحقق من صحة المدخلات.
+  3. **البناء والتسجيل في FastMCP (FastMCP Tool Registration):**
+     - دمج الدوال في خادم FastMCP موحد ومستقر مع إلزام ترميز UTF-8 ودعم التزامن `asyncio.to_thread`.
+     - تسجيل الخادم وأدواته في `mcp_config.json` للـ IDE والوكلاء.
+  4. **الأرشفة الآمنة وحماية قرص النظام (Secondary Drive Archiving):**
+     - نقل السكربتات القديمة تلقائياً إلى مجلد أرشيف منظم على القرص الثانوي (`G:\_scripts_archive` أو حسب القرص المخصص) مع حظر الحفظ على قرص النظام `C:\`.
+  5. **تحديث مهارات الوكلاء والذاكرة:**
+     - تحديث بطاقات المهارات في `.agents/skills` لتمكين الوكلاء المتخصصين من استدعاء أدوات الـ MCP الجديدة مباشرة.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>م</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>اسم الخطاف</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>المحفزات (الخطاف للنسخ)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>النموذج الأساسي والبديل</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>الوكلاء المسؤولون</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>الهدف الأساسي</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>الوصف والتفاصيل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>24. خطاف أتمتة مسارات العمل ووكلاء n8n الذكية</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ابني مسار n8n, أتمتة n8n, وكيل n8n, n8n ai agent, n8n workflow, تصميم ورك فلو</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Gemini 3.7 Flash (High)`</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>[n8n-ai-agent-architect], [mcp-tool-builder], [backend-architect], [agent-optimizer]</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>تصميم وبناء مسارات عمل ذكية مؤتمتة على n8n، ربط الوكلاء المتعددين (Multi-Agent Sub-workflows)، تتبع التحويلات وتأهيل العملاء، وربط خوادم MCP وقواعد البيانات الموجهة بالذكاء الاصطناعي.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>* **طريقة العمل والإجراءات:**
+  1. **التصميم المعماري للمسار (`n8n-ai-agent-architect`):**
+     - اختيار النمط المعماري المناسب (Multi-Agent Router, ReAct Tools Agent, Evaluator-Optimizer Loop, أو Human-in-the-Loop).
+  2. **بناء وهيكلة أدوات الاستدعاء (Tool Calling &amp; JSON Schemas):**
+     - بناء وتوثيق أدوات HTTP Request و Custom JavaScript Tools مع فرض JSON Schema صارم يمنع هلوسة المعاملات.
+  3. **إدارة طبقات الذاكرة (Short-Term &amp; Vector Memory):**
+     - ربط الذاكرة القصيرة (Window Buffer) والذاكرة المستمرة (Postgres/Redis) ومخازن المتجهات الدلالية (Qdrant/Pinecone/Supabase).
+  4. **أتمتة العمليات التسويقية وتأهيل العملاء (Marketing &amp; CRM Pipelines):**
+     - بناء مسارات استقبال وتحليل بيانات العملاء المحتملين من Google Ads و Facebook وتوجيه الإشعارات اللحظية عبر WhatsApp و Slack وتحديث الـ CRM.
+  5. **تحصين الانقطاع ومعالجة الأخطاء (Fault Tolerance &amp; Sub-workflow Retries):**
+     - إضافة مسارات الخطأ (Error Trigger) وإعادة المحاولة مع التراجع التلقائي (Exponential Backoff) ونماذج LLM البديلة.
 &lt;/div&gt;</t>
         </is>
       </c>
@@ -2789,12 +3341,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>3. خطاف الإشراف العام وتصحيح المسار</t>
+          <t>3. خطاف التخصيص والتصدير الذكي لطاقم المشروع</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
+          <t>اعتمد سياق المشروع, تخصيص وكلاء المشروع, تصدير بيئة المشروع, تخصيص الوكلاء</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2805,21 +3357,21 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[prompt-engineer], [agent-optimizer]</t>
+          <t>[code-architect], [agent-optimizer], [prompt-engineer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تصحيح الخطافات الخاطئة والبرومبتات غير الاحترافية وتوجيهها للمسار الصحيح تلقائياً.</t>
+          <t>تحليل سياق المشروع وتصدير حزم الوكلاء محلياً مع التنظيف التلقائي (Pruning) وتوليد سكربت المزامنة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **الرصد التلقائي والإيقاف:** يقوم الوكيل الرئيسي بمراقبة المحادثة. عند استخدام المستخدم لمحفز "تصحيح مسار"، أو عند رصد دخول وكيل في دائرة مفرغة، يتم اعتراض العمل وإيقافه فوراً.
-  2. **التشريح الاستباقي الصارم (Prompt Autopsy &amp; Root-Cause Analysis):** يُمنع على `prompt-engineer` تقديم برومبت جديد مباشرة. يجب أولاً طباعة قسم `[ROOT-CAUSE ANALYSIS]` يشرح بوضوح سبب الانحراف السابق (هلوسة وكيل، غياب سياق، أو معمارية خاطئة).
-  3. **حماية السياق (Context Preservation):** تحديد المتطلبات أو الملفات التي كانت تنقص الوكيل السابق للعمل بشكل صحيح تحت قسم `[MISSING ARTIFACTS / INFO]`.
-  4. **إعادة الصياغة والتوجيه القاطع (Explicit Rerouting):** توليد التوجيه الهندسي الجديد تحت قسم `[RE-ENGINEERED PROMPT]` مقترناً بشكل صريح بالوكيل الفرعي المستهدف `[TARGET HOOK]` الذي سيستلم المهمة ليكملها بنظافة.</t>
+  1. **تحليل سياق المشروع المعتمد (`project_agent_tailor.py`):** فحص ملف `PROJECT_CONTEXT.md` واكتشاف حزم التقنيات المستخدمة (مثل: `android_compose`, `web`, `python_ai`, `construction_survey`).
+  2. **تصدير حزم الوكلاء والمهارات المطلوبة:** نسخ مهارات وبطاقات الوكلاء المتخصصين وحزمة النواة حصرياً إلى مجلد المشروع المحلي `.agents/`.
+  3. **التنظيف التلقائي الصارم للمهارات الفائضة (Pruning Engine):** مسح وحذف أي مهارات أو بطاقات وكلاء غير مستخدمة في المشروع المستهدف، لحماية نافذة السياق (Context Budget) من الهدر بنسبة 100%.
+  4. **توليد قالب المزامنة المحلي (`sync_local_agents.py`):** إنشاء سكربت خفيف داخل المشروع لتمكين المطور من تحديث طاقم المشروع بنقرة زر واحدة مستقبلاً دون المساس بخصوصية المشروع.</t>
         </is>
       </c>
     </row>
@@ -2889,39 +3441,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>4. خطاف خط الإنتاج البرمجي</t>
+          <t>4. خطاف الإشراف العام وتصحيح المسار</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
+          <t>تصحيح مسار, تعديل البرومبت, خطأ بالخطاف, تصحيح خطاف</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+ البديل: `Gemini 3.7 Flash (High)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-architect], [android-kotlin-pro], [jetpack-compose-ui], [code-reviewer-quality], [clean-code-guard], [android-testing], [test-guard]</t>
+          <t>[prompt-engineer], [agent-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>تنفيذ دورة التطوير الكاملة (المعمارية، البرمجة، حراسة الكود النظيف، والفحص والاختبار).</t>
+          <t>تصحيح الخطافات الخاطئة والبرومبتات غير الاحترافية وتوجيهها للمسار الصحيح تلقائياً.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  0. **حقن السياق الإجباري (Mandatory Context Injection):** يُلزم الوكيل الرئيسي بتشغيل أداة حقن السياق (`python .agents/inject_context.py`) وتمرير مخرجاتها كـ `System Alert` أو `&gt; [!WARNING] Mandatory Constraints` في المحادثة قبل بدء أي عمل.
-  1. **التصميم المعماري الهيكلي (`code-architect`):** يبدأ برسم معمارية الميزة وتحديد مواقع وتسمية الملفات الجديدة/المعدلة في الهيكل المناسب (Data/Domain/UI).
-  2. **التدقيق المعماري الصارم وحلقة الـ 7 مرات (7-Iterations Devil's Advocate Loop):** يُمنع منعاً باتاً البدء بكتابة الكود. يجب إدخال خطة التنفيذ (`implementation_plan.md`) في حلقة مراجعة وتدقيق مع "محامي الشيطان" **لـ 7 مرات متتالية** حتى يتم سد كل الثغرات والوصول لنسبة نجاح 99.99% وتأمين قسم `[UNINTENDED SIDE-EFFECTS &amp; LIFECYCLE HAZARDS]` بالكامل قبل السماح بالكتابة.
-  3. **الكتابة البرمجية (Surgical Precision Execution):** يستلم الوكيل `[android-kotlin-pro]` أو `[jetpack-compose-ui]` الخطة المعتمدة ويبدأ بالتنفيذ. **يُحقن الوكيل بالبرومبت الإجباري التالي:** *(يُمنع منعاً باتاً المساس، أو تعديل، أو حذف أي كود حالي في المشروع لا ينص عليه صراحة في خطة التنفيذ. تصرف كجراح دقيق: أضف ميزتك فقط دون إحداث أي تغييرات جانبية في الملفات المفتوحة).*
-  4. **المراجعة وحراسة الكود النظيف (`code-reviewer-quality` + `clean-code-guard`):** يفحص الكود بعد كتابته للتحقق من الاتساق، وخلوه من أخطاء الـ AI الـ 14 الشائعة (ابتلاع الأخطاء، تضخم الدوال، الأكواد المكررة).
-  5. **الأتمتة والاختبار النظيف (`android-testing` + `test-guard`):** ينهي الدورة بكتابة وتشغيل اختبارات الوحدة (JUnit/MockK) وفق معايير `test-guard` للتحقق من سلوك النظام الفعلي وليس فقط الـ Happy Path، وتجنب الـ Mocks المفرطة.</t>
+  1. **الرصد التلقائي والإيقاف:** يقوم الوكيل الرئيسي بمراقبة المحادثة. عند استخدام المستخدم لمحفز "تصحيح مسار"، أو عند رصد دخول وكيل في دائرة مفرغة، يتم اعتراض العمل وإيقافه فوراً.
+  2. **التشريح الاستباقي الصارم (Prompt Autopsy &amp; Root-Cause Analysis):** يُمنع على `prompt-engineer` تقديم برومبت جديد مباشرة. يجب أولاً طباعة قسم `[ROOT-CAUSE ANALYSIS]` يشرح بوضوح سبب الانحراف السابق (هلوسة وكيل، غياب سياق، أو معمارية خاطئة).
+  3. **حماية السياق (Context Preservation):** تحديد المتطلبات أو الملفات التي كانت تنقص الوكيل السابق للعمل بشكل صحيح تحت قسم `[MISSING ARTIFACTS / INFO]`.
+  4. **إعادة الصياغة والتوجيه القاطع (Explicit Rerouting):** توليد التوجيه الهندسي الجديد تحت قسم `[RE-ENGINEERED PROMPT]` مقترناً بشكل صريح بالوكيل الفرعي المستهدف `[TARGET HOOK]` الذي سيستلم المهمة ليكملها بنظافة.</t>
         </is>
       </c>
     </row>
@@ -2991,37 +3541,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>5. خطاف التكامل الفني</t>
+          <t>5. خطاف خط الإنتاج البرمجي</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ربط API, تكامل خارجي</t>
+          <t>ابدأ ميزة, تطوير ميزة, اصنع ميزة, إصلاح ميزة</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Claude Sonnet 4.6 (Thinking)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[devops-deployer], [backend-architect]</t>
+          <t>[code-architect], [ui-ux-pro-max], [clean-code-guard], [test-guard]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
+          <t>تنفيذ دورة التطوير الكاملة (المعمارية، الذكاء التصميمي، البرمجة، حراسة الكود النظيف، والفحص والاختبار).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
-  2. **تحصين الانقطاع (API FAULT TOLERANCE CHECK):** يُمنع الدمج دون بناء `Interceptor` لمعالجة انقطاع الشبكة وإعادة المحاولة (Retry Mechanism)، وتغليف الردود بـ `Result&lt;T&gt;` أو `ErrorMapper` لمعالجة أخطاء HTTP (401, 404, 500).
-  3. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع وضمان التخزين المؤقت (Offline-First).
-  4. **حماية البيئة:** التأكد من عدم كتابة أي كود يحتوي على مفاتيح سرية (API Keys) في مستودع الكود وتخزينها في متغيرات البيئة فقط.</t>
+  1. **التصميم الهيكلي والذكاء التصميمي (`code-architect` + `ui-ux-pro-max`):** تحديد المعمارية المناسبة، واستدعاء محرك الاستدلال التصميمي لتحديد نمط الواجهات (Style)، باليت الألوان الدلالية، والخطوط وقواعد سهولة الوصول بدقة قبل كتابة أي واجهة.
+  2. **التدقيق المعماري الصارم (Devil's Advocate Audit):** مراجعة الخطة وكشف الثغرات وحالات الحافة لمنع الآثار الجانبية.
+  3. **الكتابة البرمجية والتنفيذ:** كتابة الكود وبناء الواجهات وقواعد البيانات محلياً.
+  4. **المراجعة وضمان الجودة (`clean-code-guard` + `test-guard`):** فحص الكود للأمان، الأداء، والتوافق مع المعايير.</t>
         </is>
       </c>
     </row>
@@ -3091,36 +3641,36 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>6. خطاف تدقيق الصيانة</t>
+          <t>6. خطاف التكامل الفني</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تدقيق صيانة, مراجعة DRY, كود نظيف</t>
+          <t>ربط API, تكامل خارجي</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Gemini 3.7 Flash (High)`</t>
+          <t>الأساسي: `Gemini 3.7 Flash (High)` 
+ البديل: `Claude Sonnet 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[code-reviewer-quality], [clean-code-guard], [performance-optimizer]</t>
+          <t>[devops-deployer], [backend-architect]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية وتطبيق معايير الكود النظيف.</t>
+          <t>ربط وتكامل الخدمات الخارجية بعد مراجعة وثائقها الرسمية وتأمين المتغيرات.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص الكود النظيف والمكرر:** استدعاء الوكيل `[code-reviewer-quality]` و `[clean-code-guard]` لمسح الملفات والتحقق من عدم وجود دوال أو منطق مكرر (تطبيق مبدأ DRY/KISS/YAGNI) والحد من التعقيد الحسابي.
-  2. **فحص Recomposition والأداء:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.
-  3. **إنشاء تقرير Refactoring:** تزويد المطور بقائمة تعديلات مقترحة لتسهيل القراءة وضغط الكود وحذف الأكواد الميتة (Dead Code).</t>
+  1. **قراءة الوثائق:** يقرأ الوكيل `[devops-deployer]` وثائق الـ API الخارجية الرسمية المدخلة قبل البدء بالدمج.
+  2. **تحصين الانقطاع (API FAULT TOLERANCE CHECK):** بناء Interceptor لمعالجة انقطاع الشبكة وإعادة المحاولة وتأمين المفاتيح في متغيرات البيئة.
+  3. **توليد الـ Wrapper:** عزل منطق التكامل في كلاسات مغلفة منفصلة لتجنب تشتيت الكود الأساسي للمشروع.</t>
         </is>
       </c>
     </row>
@@ -3190,36 +3740,35 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>7. خطاف الفحص الأمني</t>
+          <t>7. خطاف تدقيق الصيانة</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>فحص أمني, مراجعة أمان</t>
+          <t>تدقيق صيانة, مراجعة DRY, كود نظيف</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
- البديل: `Claude Opus 4.6 (Thinking)`</t>
+ البديل: `Gemini 3.7 Flash (High)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[security-auditor], [code-reviewer-quality]</t>
+          <t>[code-reviewer-quality], [clean-code-guard], [performance-optimizer]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
+          <t>مراجعة الكود البرمجي بانتظام لمنع التكرار وتراكم الديون التقنية وتطبيق معايير الكود النظيف.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest للبحث عن المكونات المكشوفة (`Exported=true`)، وتسريب البيانات عبر `Intents` (Intent Hijacking)، وقواعد `ProGuard`.
-  2. **التحقق من صحة المدخلات:** التأكد من وجود معالجة وفحص صريح لكل المدخلات والطلبات الخارجية قبل تمريرها لطبقة البيانات.
-  3. **فحص تشفير البيانات:** التحقق من تشفير البيانات الحساسة و `SharedPreferences` والجلسات وحمايتها محلياً وسحابياً (إلزام إخراج تقرير يؤكد الفحص).</t>
+  1. **فحص الكود النظيف والمكرر:** استدعاء الوكيل `[code-reviewer-quality]` و `[clean-code-guard]` لمسح الملفات والتحقق من عدم وجود دوال مكررة (تطبيق DRY/KISS/YAGNI).
+  2. **فحص Recomposition والأداء:** قياس كفاءة الرسم وإعاقات الأداء في Compose بواسطة `[performance-optimizer]`.</t>
         </is>
       </c>
     </row>
@@ -3289,44 +3838,35 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>8. خطاف مراجعة وتحديث المكتبات والنماذج</t>
+          <t>8. خطاف الفحص الأمني</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>تحديث الاعتماديات, تحديث المكتبات, تحديث النماذج, معايرة النماذج, update models</t>
+          <t>فحص أمني, مراجعة أمان</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>الأساسي: `Gemini 3.7 Flash (High)` 
- البديل: `Gemini 3.6 Flash (Medium)`</t>
+          <t>الأساسي: `Claude Sonnet 4.6 (Thinking)` 
+ البديل: `Claude Opus 4.6 (Thinking)`</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[github-talent-scout], [code-architect], [agent-optimizer]</t>
+          <t>[security-auditor], [code-reviewer-quality]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>فحص ملفات Gradle وتحديث المكتبات، والتحقق التلقائي عبر الإنترنت (antigravity.google) لتحديث مصفوفة النماذج ودليل hooks_user_guide.md دون لقطات شاشة.</t>
+          <t>مراجعة ثغرات الأمان والتحقق من صحة المدخلات وتشفير البيانات وتأمين الوصول.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>* **طريقة العمل والإجراءات:**
-  1. **فحص إصدارات المكتبات:** مسح ملفات `build.gradle.kts` ومقارنة إصدارات المكتبات الحالية بأحدث الإصدارات المستقرة.
-  2. **الاستكشاف والمعايرة التلقائية للنماذج عبر الإنترنت (Online Model Discovery):**
-     - عند كتابة محفز `"تحديث النماذج"` أو `"معايرة النماذج"`، يقوم الوكيل `[agent-optimizer]` بالاستعلام الفوري عبر الإنترنت من المصادر الرسمية:
-       - 🌐 بوابة Google Antigravity الرسمية: `https://antigravity.google`
-       - 🌐 مدونة مطوري جوجل: `https://google.dev` و `https://blog.google`
-       - 🌐 دليل وثائق Anthropic: `https://docs.anthropic.com`
-     - يتم استخراج قائمة النماذج الفعالة في المحرر (مثل `Gemini 3.7 Flash`, `Claude Sonnet 4.6 (Thinking)`).
-  3. **التحديث والمزامنة الشاملة:**
-     - تحديث مصفوفة النماذج في `HOOKS_GUIDE.md` ودليل مسار العمل `hooks_user_guide.md`.
-     - تشغيل السكربتات لتحديث ملف الإكسيل `HOOKS_GUIDE.xlsx` وتطبيق مكتبة الأوامر HTML.
-     - تشغيل `sync_global_ecosystem.py` ورفع التحديثات لـ GitHub تلقائياً.</t>
+  1. **مصفوفة الثغرات الصارمة (VULNERABILITY MATRIX):** مسح إجباري لـ AndroidManifest والمكونات المكشوفة وتسريب البيانات.
+  2. **التحقق من صحة المدخلات وتشفير البيانات:** فحص تشفير البيانات الحساسة والجلسات وتأمين الوصول محلياً وسحابياً.</t>
         </is>
       </c>
     </row>

</xml_diff>